<commit_message>
Change MH to CBMH in excel and civil3D image, EX CBMH
</commit_message>
<xml_diff>
--- a/calculations/187_Borden_Design_Calculations.xlsx
+++ b/calculations/187_Borden_Design_Calculations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\patel\Desktop\187-Borden-Conceptual-FSR-SWM\calculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FAD212C-AD86-424D-98B8-4B38CF01C3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1E87C8-31E6-46BB-897D-CF24F956BC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F13A522B-2C41-4D88-BFC8-2A0AACC7E2AC}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="93">
   <si>
     <t>Building</t>
   </si>
@@ -227,9 +227,6 @@
     <t>Inflow m3/s</t>
   </si>
   <si>
-    <t>Manholes</t>
-  </si>
-  <si>
     <t>Pipes</t>
   </si>
   <si>
@@ -309,6 +306,21 @@
   </si>
   <si>
     <t>AREA m2</t>
+  </si>
+  <si>
+    <t>CBMH1</t>
+  </si>
+  <si>
+    <t>CBMH2</t>
+  </si>
+  <si>
+    <t>CBMH3</t>
+  </si>
+  <si>
+    <t>CBMH4</t>
+  </si>
+  <si>
+    <t>CBMHs</t>
   </si>
 </sst>
 </file>
@@ -1414,7 +1426,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C1" t="s">
         <v>4</v>
@@ -1856,17 +1868,17 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -1891,7 +1903,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
@@ -1901,27 +1913,27 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
@@ -2420,17 +2432,17 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -2455,7 +2467,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
@@ -2465,27 +2477,27 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
@@ -3274,24 +3286,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" t="s">
         <v>64</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>65</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>66</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>67</v>
-      </c>
-      <c r="E2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -3305,59 +3317,59 @@
         <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4">
+      <c r="A4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="1">
         <v>1.2</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>1.2</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>1.95</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <f>3.14*(B4/2)^2*D4</f>
         <v>2.2042800000000002</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5">
+      <c r="A5" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="1">
         <v>1.2</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <v>1.2</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="1">
         <v>2.077</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <f t="shared" ref="E5:E7" si="0">3.14*(B5/2)^2*D5</f>
         <v>2.3478408000000002</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6">
+      <c r="A6" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" s="1">
         <v>1.2</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <v>1.2</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="1">
         <v>2.1880000000000002</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <f t="shared" si="0"/>
         <v>2.4733152000000005</v>
       </c>
@@ -3376,24 +3388,24 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" t="s">
         <v>70</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" t="s">
         <v>71</v>
       </c>
-      <c r="C13" t="s">
-        <v>65</v>
-      </c>
-      <c r="D13" t="s">
-        <v>72</v>
-      </c>
       <c r="E13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -3404,41 +3416,59 @@
         <v>38</v>
       </c>
       <c r="E14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C15">
+      <c r="A15" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" s="1">
         <v>19.5</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="1">
         <v>0.3</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="1">
         <f>(3.14*D15*D15)*C15/4</f>
         <v>1.3776749999999998</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C16">
+      <c r="A16" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C16" s="1">
         <v>16.2</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="1">
         <v>0.3</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="1">
         <f t="shared" ref="E16:E17" si="1">(3.14*D16*D16)*C16/4</f>
         <v>1.1445299999999998</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C17">
+      <c r="A17" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="1">
         <v>9.1</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="1">
         <v>0.3</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="1">
         <f t="shared" si="1"/>
         <v>0.6429149999999999</v>
       </c>
@@ -3451,88 +3481,90 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>73</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="A23" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E23" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B24" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" t="s">
-        <v>38</v>
-      </c>
-      <c r="D24" t="s">
-        <v>69</v>
-      </c>
+      <c r="E24" s="1"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25">
+      <c r="A25" s="1">
         <v>1</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="1">
         <v>26.178000000000001</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="1">
         <v>0.2</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="1">
         <f>C25*B25</f>
         <v>5.2356000000000007</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="1">
         <v>335.71</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26">
+      <c r="A26" s="1">
         <v>2</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="1">
         <v>39.405000000000001</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="1">
         <v>0.2</v>
       </c>
-      <c r="D26">
+      <c r="D26" s="1">
         <f t="shared" ref="D26:D27" si="2">C26*B26</f>
         <v>7.8810000000000002</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="1">
         <v>335.71</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27">
+      <c r="A27" s="1">
         <v>3</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="1">
         <v>23.593</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="1">
         <v>0.2</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="1">
         <f t="shared" si="2"/>
         <v>4.7186000000000003</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="1">
         <v>335.71</v>
       </c>
     </row>
@@ -3544,7 +3576,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F30">
         <f>D28+E19+E8</f>

</xml_diff>